<commit_message>
Atualizações de tempo em prol de bugs
</commit_message>
<xml_diff>
--- a/Plan_RA.xlsx
+++ b/Plan_RA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{358036D3-551A-4DD0-A395-2EB2107786EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4DDDB5-38B7-4A1D-B960-22E841BA3DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,7 +100,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -149,15 +149,6 @@
       <b/>
       <u/>
       <sz val="12"/>
-      <color rgb="FFFFFF00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="12"/>
       <color rgb="FFFFC000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -178,8 +169,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -194,7 +201,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF002060"/>
+        <fgColor rgb="FF094527"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF158D62"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -226,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -250,37 +263,52 @@
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -301,6 +329,14 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF158D62"/>
+      <color rgb="FF094527"/>
+      <color rgb="FF0E8449"/>
+      <color rgb="FF15CD4A"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -575,7 +611,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF19"/>
+  <dimension ref="A1:AF6"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="18" width="25.77734375" style="1" customWidth="1"/>
@@ -585,98 +621,98 @@
     <col min="33" max="16384" width="8.88671875" style="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="16" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:29" s="14" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="11" t="s">
+      <c r="L1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="11" t="s">
+      <c r="M1" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="N1" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="O1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="P1" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="Q1" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="R1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="S1" s="13"/>
-      <c r="T1" s="13"/>
-      <c r="U1" s="13"/>
-      <c r="V1" s="11"/>
-      <c r="W1" s="11"/>
-      <c r="X1" s="11"/>
-      <c r="Y1" s="14"/>
-      <c r="Z1" s="11"/>
-      <c r="AA1" s="11"/>
-      <c r="AB1" s="11" t="s">
+      <c r="S1" s="11"/>
+      <c r="T1" s="11"/>
+      <c r="U1" s="11"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="10"/>
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="AC1" s="15"/>
+      <c r="AC1" s="13"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="17"/>
       <c r="B2" s="17"/>
       <c r="C2" s="17"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
       <c r="S2" s="5"/>
       <c r="T2" s="5"/>
-      <c r="U2" s="9"/>
-      <c r="V2" s="10"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="9"/>
       <c r="W2" s="4"/>
       <c r="X2" s="4"/>
       <c r="Y2" s="7"/>
@@ -692,25 +728,25 @@
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
       <c r="S3" s="5"/>
       <c r="T3" s="5"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="10"/>
+      <c r="U3" s="8"/>
+      <c r="V3" s="9"/>
       <c r="W3" s="4"/>
       <c r="X3" s="4"/>
       <c r="Y3" s="7"/>
@@ -726,25 +762,25 @@
       <c r="A4" s="17"/>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="10"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="9"/>
       <c r="W4" s="4"/>
       <c r="X4" s="4"/>
       <c r="Y4" s="7"/>
@@ -756,29 +792,29 @@
       </c>
       <c r="AC4"/>
     </row>
-    <row r="5" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="4"/>
+    <row r="5" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="20"/>
       <c r="S5" s="4"/>
       <c r="T5" s="4"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="10"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="9"/>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
       <c r="Y5" s="7"/>
@@ -790,29 +826,29 @@
       </c>
       <c r="AC5"/>
     </row>
-    <row r="6" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
+    <row r="6" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
+      <c r="O6" s="20"/>
+      <c r="P6" s="20"/>
+      <c r="Q6" s="20"/>
+      <c r="R6" s="20"/>
       <c r="S6" s="4"/>
       <c r="T6" s="4"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="10"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="9"/>
       <c r="W6" s="4"/>
       <c r="X6" s="4"/>
       <c r="Y6" s="7"/>
@@ -824,470 +860,28 @@
       </c>
       <c r="AC6"/>
     </row>
-    <row r="7" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="4"/>
-      <c r="S7" s="4"/>
-      <c r="T7" s="4"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="4"/>
-      <c r="X7" s="4"/>
-      <c r="Y7" s="4"/>
-      <c r="Z7" s="4"/>
-      <c r="AA7" s="4"/>
-      <c r="AB7" s="6">
-        <f>IF(B7="",0,VLOOKUP(Z7,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC7"/>
-    </row>
-    <row r="8" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
-      <c r="R8" s="4"/>
-      <c r="S8" s="4"/>
-      <c r="T8" s="4"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="10"/>
-      <c r="W8" s="4"/>
-      <c r="X8" s="4"/>
-      <c r="Y8" s="4"/>
-      <c r="Z8" s="4"/>
-      <c r="AA8" s="4"/>
-      <c r="AB8" s="6">
-        <f>IF(B8="",0,VLOOKUP(Z8,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC8"/>
-    </row>
-    <row r="9" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="4"/>
-      <c r="S9" s="4"/>
-      <c r="T9" s="4"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="10"/>
-      <c r="W9" s="4"/>
-      <c r="X9" s="4"/>
-      <c r="Y9" s="4"/>
-      <c r="Z9" s="4"/>
-      <c r="AA9" s="4"/>
-      <c r="AB9" s="6">
-        <f>IF(B9="",0,VLOOKUP(Z9,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC9"/>
-    </row>
-    <row r="10" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="4"/>
-      <c r="S10" s="4"/>
-      <c r="T10" s="4"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="10"/>
-      <c r="W10" s="4"/>
-      <c r="X10" s="4"/>
-      <c r="Y10" s="4"/>
-      <c r="Z10" s="4"/>
-      <c r="AA10" s="4"/>
-      <c r="AB10" s="6">
-        <f>IF(B10="",0,VLOOKUP(Z10,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC10"/>
-    </row>
-    <row r="11" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
-      <c r="R11" s="4"/>
-      <c r="S11" s="4"/>
-      <c r="T11" s="4"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="10"/>
-      <c r="W11" s="4"/>
-      <c r="X11" s="4"/>
-      <c r="Y11" s="4"/>
-      <c r="Z11" s="4"/>
-      <c r="AA11" s="4"/>
-      <c r="AB11" s="6">
-        <f>IF(B11="",0,VLOOKUP(Z11,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC11"/>
-    </row>
-    <row r="12" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
-      <c r="S12" s="4"/>
-      <c r="T12" s="4"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="10"/>
-      <c r="W12" s="4"/>
-      <c r="X12" s="4"/>
-      <c r="Y12" s="4"/>
-      <c r="Z12" s="4"/>
-      <c r="AA12" s="4"/>
-      <c r="AB12" s="6">
-        <f>IF(B12="",0,VLOOKUP(Z12,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC12"/>
-    </row>
-    <row r="13" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="4"/>
-      <c r="S13" s="4"/>
-      <c r="T13" s="4"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="10"/>
-      <c r="W13" s="4"/>
-      <c r="X13" s="4"/>
-      <c r="Y13" s="4"/>
-      <c r="Z13" s="4"/>
-      <c r="AA13" s="4"/>
-      <c r="AB13" s="6">
-        <f>IF(B13="",0,VLOOKUP(Z13,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC13"/>
-    </row>
-    <row r="14" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="4"/>
-      <c r="T14" s="4"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="10"/>
-      <c r="W14" s="4"/>
-      <c r="X14" s="4"/>
-      <c r="Y14" s="4"/>
-      <c r="Z14" s="4"/>
-      <c r="AA14" s="4"/>
-      <c r="AB14" s="6">
-        <f>IF(B14="",0,VLOOKUP(Z14,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC14"/>
-    </row>
-    <row r="15" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="4"/>
-      <c r="S15" s="4"/>
-      <c r="T15" s="4"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="10"/>
-      <c r="W15" s="4"/>
-      <c r="X15" s="4"/>
-      <c r="Y15" s="4"/>
-      <c r="Z15" s="4"/>
-      <c r="AA15" s="4"/>
-      <c r="AB15" s="6">
-        <f>IF(B15="",0,VLOOKUP(Z15,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC15"/>
-    </row>
-    <row r="16" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="10"/>
-      <c r="W16" s="4"/>
-      <c r="X16" s="4"/>
-      <c r="Y16" s="4"/>
-      <c r="Z16" s="4"/>
-      <c r="AA16" s="4"/>
-      <c r="AB16" s="6">
-        <f>IF(B16="",0,VLOOKUP(Z16,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC16"/>
-    </row>
-    <row r="17" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
-      <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
-      <c r="R17" s="4"/>
-      <c r="S17" s="4"/>
-      <c r="T17" s="4"/>
-      <c r="U17" s="9"/>
-      <c r="V17" s="10"/>
-      <c r="W17" s="4"/>
-      <c r="X17" s="4"/>
-      <c r="Y17" s="4"/>
-      <c r="Z17" s="4"/>
-      <c r="AA17" s="4"/>
-      <c r="AB17" s="6">
-        <f>IF(B17="",0,VLOOKUP(Z17,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC17"/>
-    </row>
-    <row r="18" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
-      <c r="R18" s="4"/>
-      <c r="S18" s="4"/>
-      <c r="T18" s="4"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="10"/>
-      <c r="W18" s="4"/>
-      <c r="X18" s="4"/>
-      <c r="Y18" s="4"/>
-      <c r="Z18" s="4"/>
-      <c r="AA18" s="4"/>
-      <c r="AB18" s="6">
-        <f>IF(B18="",0,VLOOKUP(Z18,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC18"/>
-    </row>
-    <row r="19" spans="1:29" s="3" customFormat="1" ht="19.95" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4"/>
-      <c r="O19" s="4"/>
-      <c r="P19" s="4"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="4"/>
-      <c r="S19" s="4"/>
-      <c r="T19" s="4"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="10"/>
-      <c r="W19" s="4"/>
-      <c r="X19" s="4"/>
-      <c r="Y19" s="4"/>
-      <c r="Z19" s="4"/>
-      <c r="AA19" s="4"/>
-      <c r="AB19" s="6">
-        <f>IF(B19="",0,VLOOKUP(Z19,Planilha1!#REF!,2,FALSE))</f>
-        <v>0</v>
-      </c>
-      <c r="AC19"/>
-    </row>
   </sheetData>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="K1 K5:M1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W5:W19" xr:uid="{AEBEAE45-30D1-4542-A1D6-EBC88D16BDC1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W5:W6" xr:uid="{AEBEAE45-30D1-4542-A1D6-EBC88D16BDC1}">
       <formula1>"KG, L, Ds"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA5:AB19" xr:uid="{515AD032-001C-4B14-8366-B098E8D106E9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA5:AB6" xr:uid="{515AD032-001C-4B14-8366-B098E8D106E9}">
       <formula1>"NITRO, FORNECEDOR, DEVOLUÇÃO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X5:X19" xr:uid="{9224D280-D2F8-4702-BD9E-3A2E00F78617}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X5:X6" xr:uid="{9224D280-D2F8-4702-BD9E-3A2E00F78617}">
       <formula1>"Saco, Bombona, Palete, Caixa, Big Bag, Galão"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I19" xr:uid="{0CCEE7D2-5A92-4296-95B7-680EA05B05B1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I6" xr:uid="{0CCEE7D2-5A92-4296-95B7-680EA05B05B1}">
       <formula1>"VZP TRANSF HORT, DEVOLUÇÃO CLIENTE, VZP TRANSF CBA, RECEBIMENTO PORTO, ROO TRANSF HORT, ROO TRANSF CBA, HORT TRANSF CBA, TORRE DE CONTROLE, TRANSP. RODOFROTA, STZ TRANSF HORT, CBA TRANSF HORT, STZ TRANSF CBA, FORNECEDOR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I19 G5:G19" xr:uid="{A9DDEBF6-CC05-4C4C-B66F-05CC7D4CAF45}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I6 G5:G6" xr:uid="{A9DDEBF6-CC05-4C4C-B66F-05CC7D4CAF45}">
       <formula1>"Cuiabá, Hortolândia"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5:J19" xr:uid="{EE69AD02-7E08-441A-857C-3BD9A1515FF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5:J6" xr:uid="{EE69AD02-7E08-441A-857C-3BD9A1515FF8}">
       <formula1>"FORNECEDOR, DEVOLUÇÃO CLIENTE, VZP NITRO, HORT, CUIABÁ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F4" xr:uid="{1FA120A8-14C6-4F7D-BB1D-E2BEE940ECF5}">
@@ -1318,7 +912,7 @@
           <x14:formula1>
             <xm:f>Planilha1!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>Z5:Z19</xm:sqref>
+          <xm:sqref>Z5:Z6</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Atualização de tempos de espera e correção de bugs
</commit_message>
<xml_diff>
--- a/Plan_RA.xlsx
+++ b/Plan_RA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E4DDDB5-38B7-4A1D-B960-22E841BA3DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2608E31C-995D-49BD-AD8F-CF18D80D7C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>PASTA-ANEXOS</t>
   </si>
@@ -94,6 +94,54 @@
   </si>
   <si>
     <t>TIPO-EMBALAGEM</t>
+  </si>
+  <si>
+    <t>Rasgada /Amassada</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>Sacaria</t>
+  </si>
+  <si>
+    <t>117</t>
+  </si>
+  <si>
+    <t>ra-01</t>
+  </si>
+  <si>
+    <t>MMCM - HOR</t>
+  </si>
+  <si>
+    <t>Expedição - Carregamento</t>
+  </si>
+  <si>
+    <t>5283</t>
+  </si>
+  <si>
+    <t>SPEED CITROS SCX25KG</t>
+  </si>
+  <si>
+    <t>05026</t>
+  </si>
+  <si>
+    <t>6925935</t>
+  </si>
+  <si>
+    <t>59691/24</t>
+  </si>
+  <si>
+    <t>01/10/2024</t>
+  </si>
+  <si>
+    <t>01/10/2026</t>
+  </si>
+  <si>
+    <t>Durante o processo de carregamento, foi identificada a seguinte Avaria: A) O produto SPEED CITROS SCX25KG (NF 5283, Lote 59691/24) apresentou 25kg avariados (1 saco). No momento da estiva/movimentação para o veículo, a sacaria foi rasgada, comprometendo a integridade da embalagem e impossibilitando o envio ao cliente. O volume foi retirado da carga para segregação e posterior processo de bloqueio e recondicionamento.</t>
+  </si>
+  <si>
+    <t>Leonardo</t>
   </si>
 </sst>
 </file>
@@ -239,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -292,23 +340,27 @@
     <xf numFmtId="49" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -316,7 +368,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -611,14 +673,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF6"/>
+  <dimension ref="A1:AC6"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="18" width="25.77734375" style="1" customWidth="1"/>
-    <col min="19" max="28" width="25.77734375" style="1" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="0" hidden="1" customWidth="1"/>
-    <col min="30" max="32" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.88671875" style="1" hidden="1"/>
+    <col min="19" max="28" width="25.77734375" style="1" hidden="1"/>
+    <col min="29" max="29" width="25.77734375" hidden="1"/>
+    <col min="30" max="16384" width="25.77734375" style="1" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" s="14" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -691,24 +752,60 @@
       <c r="AC1" s="13"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
+      <c r="A2" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="N2" s="22">
+        <v>25</v>
+      </c>
+      <c r="O2" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="P2" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q2" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="18" t="s">
+        <v>34</v>
+      </c>
       <c r="S2" s="5"/>
       <c r="T2" s="5"/>
       <c r="U2" s="8"/>
@@ -720,7 +817,7 @@
       <c r="AA2" s="4"/>
       <c r="AB2" s="6">
         <f>IF(B2="",0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC2"/>
     </row>
@@ -738,7 +835,7 @@
       <c r="K3" s="18"/>
       <c r="L3" s="18"/>
       <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
+      <c r="N3" s="22"/>
       <c r="O3" s="18"/>
       <c r="P3" s="18"/>
       <c r="Q3" s="18"/>
@@ -772,7 +869,7 @@
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
+      <c r="N4" s="22"/>
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
       <c r="Q4" s="18"/>
@@ -802,11 +899,11 @@
       <c r="G5" s="20"/>
       <c r="H5" s="20"/>
       <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
+      <c r="J5" s="18"/>
       <c r="K5" s="20"/>
       <c r="L5" s="20"/>
       <c r="M5" s="20"/>
-      <c r="N5" s="21"/>
+      <c r="N5" s="22"/>
       <c r="O5" s="21"/>
       <c r="P5" s="21"/>
       <c r="Q5" s="21"/>
@@ -840,7 +937,7 @@
       <c r="K6" s="20"/>
       <c r="L6" s="20"/>
       <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
+      <c r="N6" s="22"/>
       <c r="O6" s="20"/>
       <c r="P6" s="20"/>
       <c r="Q6" s="20"/>
@@ -861,9 +958,13 @@
       <c r="AC6"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="J1:J1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K1 K5:M1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <dataValidations count="12">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W5:W6" xr:uid="{AEBEAE45-30D1-4542-A1D6-EBC88D16BDC1}">
@@ -881,7 +982,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I6 G5:G6" xr:uid="{A9DDEBF6-CC05-4C4C-B66F-05CC7D4CAF45}">
       <formula1>"Cuiabá, Hortolândia"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5:J6" xr:uid="{EE69AD02-7E08-441A-857C-3BD9A1515FF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J6" xr:uid="{EE69AD02-7E08-441A-857C-3BD9A1515FF8}">
       <formula1>"FORNECEDOR, DEVOLUÇÃO CLIENTE, VZP NITRO, HORT, CUIABÁ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F4" xr:uid="{1FA120A8-14C6-4F7D-BB1D-E2BEE940ECF5}">

</xml_diff>

<commit_message>
Módulo de RNC Múltiplas + Correção de bugs
</commit_message>
<xml_diff>
--- a/Plan_RA.xlsx
+++ b/Plan_RA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2608E31C-995D-49BD-AD8F-CF18D80D7C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C00724-B11D-4B7A-86F1-46231C8E88E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -243,12 +243,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF094527"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -256,6 +250,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF158D62"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -287,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -319,39 +319,31 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -361,6 +353,46 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -673,11 +705,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC6"/>
+  <dimension ref="A1:AC13"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="18" width="25.77734375" style="1" customWidth="1"/>
-    <col min="19" max="28" width="25.77734375" style="1" hidden="1"/>
+    <col min="19" max="28" width="0" style="1" hidden="1" customWidth="1"/>
     <col min="29" max="29" width="25.77734375" hidden="1"/>
     <col min="30" max="16384" width="25.77734375" style="1" hidden="1"/>
   </cols>
@@ -752,58 +784,58 @@
       <c r="AC1" s="13"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="N2" s="22">
+      <c r="N2" s="20">
         <v>25</v>
       </c>
-      <c r="O2" s="18" t="s">
+      <c r="O2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" s="18" t="s">
+      <c r="Q2" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="R2" s="18" t="s">
+      <c r="R2" s="17" t="s">
         <v>34</v>
       </c>
       <c r="S2" s="5"/>
@@ -822,24 +854,24 @@
       <c r="AC2"/>
     </row>
     <row r="3" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="17"/>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="18"/>
+      <c r="A3" s="30"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="17"/>
+      <c r="K3" s="17"/>
+      <c r="L3" s="17"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="17"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="17"/>
+      <c r="R3" s="17"/>
       <c r="S3" s="5"/>
       <c r="T3" s="5"/>
       <c r="U3" s="8"/>
@@ -856,24 +888,24 @@
       <c r="AC3"/>
     </row>
     <row r="4" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
       <c r="S4" s="5"/>
       <c r="T4" s="5"/>
       <c r="U4" s="8"/>
@@ -890,26 +922,26 @@
       <c r="AC4"/>
     </row>
     <row r="5" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="19"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
+      <c r="A5" s="30"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
       <c r="U5" s="8"/>
       <c r="V5" s="9"/>
       <c r="W5" s="4"/>
@@ -918,44 +950,282 @@
       <c r="Z5" s="4"/>
       <c r="AA5" s="4"/>
       <c r="AB5" s="6">
-        <f>IF(B5="",0,VLOOKUP(Z5,Planilha1!#REF!,2,FALSE))</f>
+        <f t="shared" ref="AB5:AB12" si="0">IF(B5="",0,1)</f>
         <v>0</v>
       </c>
       <c r="AC5"/>
     </row>
-    <row r="6" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="19"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
+    <row r="6" spans="1:29" s="29" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
       <c r="N6" s="22"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="8"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="7"/>
-      <c r="Z6" s="4"/>
-      <c r="AA6" s="4"/>
-      <c r="AB6" s="6">
-        <f>IF(B6="",0,VLOOKUP(Z6,Planilha1!#REF!,2,FALSE))</f>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="23"/>
+      <c r="T6" s="23"/>
+      <c r="U6" s="24"/>
+      <c r="V6" s="25"/>
+      <c r="W6" s="26"/>
+      <c r="X6" s="26"/>
+      <c r="Y6" s="27"/>
+      <c r="Z6" s="26"/>
+      <c r="AA6" s="26"/>
+      <c r="AB6" s="26">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="AC6"/>
+      <c r="AC6" s="28"/>
+    </row>
+    <row r="7" spans="1:29" s="29" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="23"/>
+      <c r="T7" s="23"/>
+      <c r="U7" s="24"/>
+      <c r="V7" s="25"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="26"/>
+      <c r="Y7" s="27"/>
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26"/>
+      <c r="AB7" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC7" s="28"/>
+    </row>
+    <row r="8" spans="1:29" s="29" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="21"/>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="23"/>
+      <c r="T8" s="23"/>
+      <c r="U8" s="24"/>
+      <c r="V8" s="25"/>
+      <c r="W8" s="26"/>
+      <c r="X8" s="26"/>
+      <c r="Y8" s="27"/>
+      <c r="Z8" s="26"/>
+      <c r="AA8" s="26"/>
+      <c r="AB8" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC8" s="28"/>
+    </row>
+    <row r="9" spans="1:29" s="29" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="21"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="23"/>
+      <c r="T9" s="23"/>
+      <c r="U9" s="24"/>
+      <c r="V9" s="25"/>
+      <c r="W9" s="26"/>
+      <c r="X9" s="26"/>
+      <c r="Y9" s="27"/>
+      <c r="Z9" s="26"/>
+      <c r="AA9" s="26"/>
+      <c r="AB9" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC9" s="28"/>
+    </row>
+    <row r="10" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="30"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="17"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="17"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="9"/>
+      <c r="W10" s="4"/>
+      <c r="X10" s="4"/>
+      <c r="Y10" s="7"/>
+      <c r="Z10" s="4"/>
+      <c r="AA10" s="4"/>
+      <c r="AB10" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC10"/>
+    </row>
+    <row r="11" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="30"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="17"/>
+      <c r="M11" s="17"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="17"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="5"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="9"/>
+      <c r="W11" s="4"/>
+      <c r="X11" s="4"/>
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="4"/>
+      <c r="AA11" s="4"/>
+      <c r="AB11" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC11"/>
+    </row>
+    <row r="12" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="31"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="20"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="18"/>
+      <c r="S12" s="4"/>
+      <c r="T12" s="4"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="9"/>
+      <c r="W12" s="4"/>
+      <c r="X12" s="4"/>
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="4"/>
+      <c r="AA12" s="4"/>
+      <c r="AB12" s="6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC12"/>
+    </row>
+    <row r="13" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="31"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
+      <c r="M13" s="18"/>
+      <c r="N13" s="20"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
+      <c r="R13" s="18"/>
+      <c r="S13" s="4"/>
+      <c r="T13" s="4"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="9"/>
+      <c r="W13" s="4"/>
+      <c r="X13" s="4"/>
+      <c r="Y13" s="7"/>
+      <c r="Z13" s="4"/>
+      <c r="AA13" s="4"/>
+      <c r="AB13" s="6">
+        <f>IF(B13="",0,VLOOKUP(Z13,Planilha1!#REF!,2,FALSE))</f>
+        <v>0</v>
+      </c>
+      <c r="AC13"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
@@ -963,44 +1233,44 @@
   <conditionalFormatting sqref="J1:J1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1 K5:M1048576">
+  <conditionalFormatting sqref="K12:M1048576 K1">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W5:W6" xr:uid="{AEBEAE45-30D1-4542-A1D6-EBC88D16BDC1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W12:W13" xr:uid="{AEBEAE45-30D1-4542-A1D6-EBC88D16BDC1}">
       <formula1>"KG, L, Ds"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA5:AB6" xr:uid="{515AD032-001C-4B14-8366-B098E8D106E9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AA12:AA13 AB13" xr:uid="{515AD032-001C-4B14-8366-B098E8D106E9}">
       <formula1>"NITRO, FORNECEDOR, DEVOLUÇÃO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X5:X6" xr:uid="{9224D280-D2F8-4702-BD9E-3A2E00F78617}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X12:X13" xr:uid="{9224D280-D2F8-4702-BD9E-3A2E00F78617}">
       <formula1>"Saco, Bombona, Palete, Caixa, Big Bag, Galão"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I6" xr:uid="{0CCEE7D2-5A92-4296-95B7-680EA05B05B1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I12:I13" xr:uid="{0CCEE7D2-5A92-4296-95B7-680EA05B05B1}">
       <formula1>"VZP TRANSF HORT, DEVOLUÇÃO CLIENTE, VZP TRANSF CBA, RECEBIMENTO PORTO, ROO TRANSF HORT, ROO TRANSF CBA, HORT TRANSF CBA, TORRE DE CONTROLE, TRANSP. RODOFROTA, STZ TRANSF HORT, CBA TRANSF HORT, STZ TRANSF CBA, FORNECEDOR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I6 G5:G6" xr:uid="{A9DDEBF6-CC05-4C4C-B66F-05CC7D4CAF45}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I12:I13 G12:G13" xr:uid="{A9DDEBF6-CC05-4C4C-B66F-05CC7D4CAF45}">
       <formula1>"Cuiabá, Hortolândia"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J6" xr:uid="{EE69AD02-7E08-441A-857C-3BD9A1515FF8}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J13" xr:uid="{EE69AD02-7E08-441A-857C-3BD9A1515FF8}">
       <formula1>"FORNECEDOR, DEVOLUÇÃO CLIENTE, VZP NITRO, HORT, CUIABÁ"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F4" xr:uid="{1FA120A8-14C6-4F7D-BB1D-E2BEE940ECF5}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F11" xr:uid="{1FA120A8-14C6-4F7D-BB1D-E2BEE940ECF5}">
       <formula1>"Conferência, Movimentação Interna ou armazenagem, Separação, Expedição - Carregamento"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O4" xr:uid="{484497D8-42F2-4C49-A4D8-BA5B5AF75B7A}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O2:O11" xr:uid="{484497D8-42F2-4C49-A4D8-BA5B5AF75B7A}">
       <formula1>"KG, L"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D4" xr:uid="{D2B05375-3588-42D9-8BB7-56B59A51B1EE}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D11" xr:uid="{D2B05375-3588-42D9-8BB7-56B59A51B1EE}">
       <formula1>"MMCM - HOR, MMCM - CBA"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E4" xr:uid="{41EB2888-F11E-456C-A00B-F6AF89D6614F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E11" xr:uid="{41EB2888-F11E-456C-A00B-F6AF89D6614F}">
       <formula1>"MMCM - HOR, MMCM - CBA, NITRO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A4" xr:uid="{2E0B6B3D-1179-4B3F-8778-41DC49DAEC8D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A11" xr:uid="{2E0B6B3D-1179-4B3F-8778-41DC49DAEC8D}">
       <formula1>"Rasgada /Amassada, Vazando"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P4" xr:uid="{63B1DB81-B8D8-4975-B6A0-4F650D7213C9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P11" xr:uid="{63B1DB81-B8D8-4975-B6A0-4F650D7213C9}">
       <formula1>"Sacaria, Bombona, Embalagem molhada, Válvula, Galão"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1013,7 +1283,7 @@
           <x14:formula1>
             <xm:f>Planilha1!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>Z5:Z6</xm:sqref>
+          <xm:sqref>Z12:Z13</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Resolução no bug do preenchimento do Sharepoint
</commit_message>
<xml_diff>
--- a/Plan_RA.xlsx
+++ b/Plan_RA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C00724-B11D-4B7A-86F1-46231C8E88E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C16FF753-69D2-46D6-988D-876B4221DB21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t>PASTA-ANEXOS</t>
   </si>
@@ -96,52 +96,94 @@
     <t>TIPO-EMBALAGEM</t>
   </si>
   <si>
-    <t>Rasgada /Amassada</t>
-  </si>
-  <si>
-    <t>KG</t>
-  </si>
-  <si>
-    <t>Sacaria</t>
-  </si>
-  <si>
-    <t>117</t>
-  </si>
-  <si>
-    <t>ra-01</t>
-  </si>
-  <si>
     <t>MMCM - HOR</t>
   </si>
   <si>
     <t>Expedição - Carregamento</t>
   </si>
   <si>
-    <t>5283</t>
-  </si>
-  <si>
-    <t>SPEED CITROS SCX25KG</t>
-  </si>
-  <si>
-    <t>05026</t>
-  </si>
-  <si>
-    <t>6925935</t>
-  </si>
-  <si>
-    <t>59691/24</t>
-  </si>
-  <si>
-    <t>01/10/2024</t>
-  </si>
-  <si>
-    <t>01/10/2026</t>
-  </si>
-  <si>
-    <t>Durante o processo de carregamento, foi identificada a seguinte Avaria: A) O produto SPEED CITROS SCX25KG (NF 5283, Lote 59691/24) apresentou 25kg avariados (1 saco). No momento da estiva/movimentação para o veículo, a sacaria foi rasgada, comprometendo a integridade da embalagem e impossibilitando o envio ao cliente. O volume foi retirado da carga para segregação e posterior processo de bloqueio e recondicionamento.</t>
-  </si>
-  <si>
     <t>Leonardo</t>
+  </si>
+  <si>
+    <t>Vazando</t>
+  </si>
+  <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
+    <t>ra01</t>
+  </si>
+  <si>
+    <t>ra02</t>
+  </si>
+  <si>
+    <t>MMCM - CBA</t>
+  </si>
+  <si>
+    <t>Separação</t>
+  </si>
+  <si>
+    <t>7480</t>
+  </si>
+  <si>
+    <t>ARRANK CX02X05L</t>
+  </si>
+  <si>
+    <t>510052</t>
+  </si>
+  <si>
+    <t>6949523</t>
+  </si>
+  <si>
+    <t>69018/25</t>
+  </si>
+  <si>
+    <t>25/06/2027</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Galão</t>
+  </si>
+  <si>
+    <t>25/06/2024</t>
+  </si>
+  <si>
+    <t>Durante a movimentação interna para separação de pedido, foi identificada a seguinte não conformidade: A) O produto ARRANK CX02X05L (NF 7480, Lote 69018/25) apresentou avaria com perda de conteúdo, totalizando 10L (01 caixa). O volume foi imediatamente segregado para evitar a contaminação de outros paletes e destinado ao setor de bloqueio para as devidas tratativas de qualidade.</t>
+  </si>
+  <si>
+    <t>10786</t>
+  </si>
+  <si>
+    <t>GROWN 1000L</t>
+  </si>
+  <si>
+    <t>04170</t>
+  </si>
+  <si>
+    <t>6921601</t>
+  </si>
+  <si>
+    <t>75490/26</t>
+  </si>
+  <si>
+    <t>19/03/2026</t>
+  </si>
+  <si>
+    <t>19/03/2029</t>
+  </si>
+  <si>
+    <t>IBC</t>
+  </si>
+  <si>
+    <t>Marcos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Durante o processo de descarga da transferência (NF 10786), foi identificada uma não conformidade crítica de embalagem: A) O produto GROWN 1000L (Lote 75490/26) apresentou avaria grave em sua unidade de transporte (IBC). No ato do recebimento, constatou-se que o IBC estava furado, com sinais de sujidade, contaminação externa e tentativas de remendo. </t>
   </si>
 </sst>
 </file>
@@ -287,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -387,14 +429,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -710,7 +744,7 @@
   <cols>
     <col min="1" max="18" width="25.77734375" style="1" customWidth="1"/>
     <col min="19" max="28" width="0" style="1" hidden="1" customWidth="1"/>
-    <col min="29" max="29" width="25.77734375" hidden="1"/>
+    <col min="29" max="29" width="25.77734375" hidden="1" customWidth="1"/>
     <col min="30" max="16384" width="25.77734375" style="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -784,59 +818,59 @@
       <c r="AC1" s="13"/>
     </row>
     <row r="2" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="30" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>24</v>
-      </c>
       <c r="E2" s="17" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I2" s="17" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J2" s="17" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="K2" s="17" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="L2" s="17" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="M2" s="17" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="N2" s="20">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="O2" s="17" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="P2" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q2" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" s="17" t="s">
         <v>21</v>
-      </c>
-      <c r="Q2" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="R2" s="17" t="s">
-        <v>34</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="5"/>
@@ -854,24 +888,60 @@
       <c r="AC2"/>
     </row>
     <row r="3" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="30"/>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="17"/>
-      <c r="P3" s="17"/>
-      <c r="Q3" s="17"/>
-      <c r="R3" s="17"/>
+      <c r="A3" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="20">
+        <v>1000</v>
+      </c>
+      <c r="O3" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="P3" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="R3" s="17" t="s">
+        <v>47</v>
+      </c>
       <c r="S3" s="5"/>
       <c r="T3" s="5"/>
       <c r="U3" s="8"/>
@@ -883,14 +953,14 @@
       <c r="AA3" s="4"/>
       <c r="AB3" s="6">
         <f>IF(B3="",0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC3"/>
     </row>
     <row r="4" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="30"/>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
+      <c r="A4" s="17"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="17"/>
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17"/>
@@ -922,9 +992,9 @@
       <c r="AC4"/>
     </row>
     <row r="5" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
       <c r="D5" s="17"/>
       <c r="E5" s="17"/>
       <c r="F5" s="17"/>
@@ -1092,9 +1162,9 @@
       <c r="AC9" s="28"/>
     </row>
     <row r="10" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="30"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
       <c r="F10" s="17"/>
@@ -1126,9 +1196,9 @@
       <c r="AC10"/>
     </row>
     <row r="11" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="30"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>
@@ -1160,9 +1230,9 @@
       <c r="AC11"/>
     </row>
     <row r="12" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="31"/>
-      <c r="B12" s="31"/>
-      <c r="C12" s="31"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="17"/>
       <c r="E12" s="17"/>
       <c r="F12" s="17"/>
@@ -1194,9 +1264,9 @@
       <c r="AC12"/>
     </row>
     <row r="13" spans="1:29" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="31"/>
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
       <c r="D13" s="17"/>
       <c r="E13" s="17"/>
       <c r="F13" s="17"/>
@@ -1228,7 +1298,6 @@
       <c r="AC13"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="J1:J1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
@@ -1270,8 +1339,8 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A11" xr:uid="{2E0B6B3D-1179-4B3F-8778-41DC49DAEC8D}">
       <formula1>"Rasgada /Amassada, Vazando"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P11" xr:uid="{63B1DB81-B8D8-4975-B6A0-4F650D7213C9}">
-      <formula1>"Sacaria, Bombona, Embalagem molhada, Válvula, Galão"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P13" xr:uid="{64D1ACFE-3253-446E-8F2A-2CB69C1560ED}">
+      <formula1>"Sacaria, Bombona, Embalagem molhada, Válvula, Galão, IBC"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Atualizações para fornecer automação para Regina
</commit_message>
<xml_diff>
--- a/Plan_RA.xlsx
+++ b/Plan_RA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iesus.candido\Desktop\RNC-RA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B10D7141-5FD2-457A-91A7-7077D40D13E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A317590F-30E3-43A0-A236-4B99565BBE7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-3990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="56">
   <si>
     <t>PASTA-ANEXOS</t>
   </si>
@@ -99,18 +99,6 @@
     <t>MMCM - HOR</t>
   </si>
   <si>
-    <t>Expedição - Carregamento</t>
-  </si>
-  <si>
-    <t>Leonardo</t>
-  </si>
-  <si>
-    <t>Vazando</t>
-  </si>
-  <si>
-    <t>118</t>
-  </si>
-  <si>
     <t>119</t>
   </si>
   <si>
@@ -120,70 +108,103 @@
     <t>ra02</t>
   </si>
   <si>
-    <t>MMCM - CBA</t>
-  </si>
-  <si>
-    <t>Separação</t>
-  </si>
-  <si>
-    <t>7480</t>
-  </si>
-  <si>
-    <t>ARRANK CX02X05L</t>
-  </si>
-  <si>
-    <t>510052</t>
-  </si>
-  <si>
-    <t>6949523</t>
-  </si>
-  <si>
-    <t>69018/25</t>
-  </si>
-  <si>
-    <t>25/06/2027</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Galão</t>
-  </si>
-  <si>
-    <t>25/06/2024</t>
-  </si>
-  <si>
-    <t>Durante a movimentação interna para separação de pedido, foi identificada a seguinte não conformidade: A) O produto ARRANK CX02X05L (NF 7480, Lote 69018/25) apresentou avaria com perda de conteúdo, totalizando 10L (01 caixa). O volume foi imediatamente segregado para evitar a contaminação de outros paletes e destinado ao setor de bloqueio para as devidas tratativas de qualidade.</t>
-  </si>
-  <si>
-    <t>10786</t>
-  </si>
-  <si>
-    <t>GROWN 1000L</t>
-  </si>
-  <si>
-    <t>04170</t>
-  </si>
-  <si>
-    <t>6921601</t>
-  </si>
-  <si>
-    <t>75490/26</t>
-  </si>
-  <si>
-    <t>19/03/2026</t>
-  </si>
-  <si>
-    <t>19/03/2029</t>
-  </si>
-  <si>
-    <t>IBC</t>
-  </si>
-  <si>
-    <t>Marcos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Durante o processo de descarga da transferência (NF 10786), foi identificada uma não conformidade crítica de embalagem: A) O produto GROWN 1000L (Lote 75490/26) apresentou avaria grave em sua unidade de transporte (IBC). No ato do recebimento, constatou-se que o IBC estava furado, com sinais de sujidade, contaminação externa e tentativas de remendo. </t>
+    <t>Rasgada /Amassada</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>ra03</t>
+  </si>
+  <si>
+    <t>Movimentação Interna ou armazenagem</t>
+  </si>
+  <si>
+    <t>SPEED CANA SCX25KG</t>
+  </si>
+  <si>
+    <t>510002</t>
+  </si>
+  <si>
+    <t>76180/26</t>
+  </si>
+  <si>
+    <t>10962</t>
+  </si>
+  <si>
+    <t>7023066</t>
+  </si>
+  <si>
+    <t>14/04/2029</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>Sacaria</t>
+  </si>
+  <si>
+    <t>Durante movimentação interna, foi identificada a seguinte não conformidade física: A) O produto SPEED CANA SCX25KG (Lote 76180/26) apresentou avaria em 02 sacarias, totalizando 50kg. No momento da movimentação, constatou-se que as embalagens estavam rasgadas, resultando em vazamento de produto e exposição do conteúdo ao ambiente. O volume foi segregado.</t>
+  </si>
+  <si>
+    <t>Rodrigo</t>
+  </si>
+  <si>
+    <t>14/04/2026</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>ra04</t>
+  </si>
+  <si>
+    <t>10970</t>
+  </si>
+  <si>
+    <t>10966</t>
+  </si>
+  <si>
+    <t>76181/26</t>
+  </si>
+  <si>
+    <t>7023201</t>
+  </si>
+  <si>
+    <t>15/04/2026</t>
+  </si>
+  <si>
+    <t>15/04/2029</t>
+  </si>
+  <si>
+    <t>Durante movimentação interna, foi identificada a seguinte não conformidade física: A) O produto SPEED CANA SCX25KG (Lote 76181/26) apresentou avaria em 02 sacarias, totalizando 50kg. As embalagens foram identificadas como rasgadas, causando o vazamento de parte do conteúdo e comprometendo a integridade do pallet. O volume foi imediatamente segregado.</t>
+  </si>
+  <si>
+    <t>10983</t>
+  </si>
+  <si>
+    <t>76182/26</t>
+  </si>
+  <si>
+    <t>7023617</t>
+  </si>
+  <si>
+    <t>16/04/2026</t>
+  </si>
+  <si>
+    <t>16/04/2029</t>
+  </si>
+  <si>
+    <t>Durante movimentação interna, foi identificada a seguinte não conformidade física: A) O produto SPEED CANA SCX25KG (Lote 76182/26) apresentou avaria em 01 sacaria, totalizando 25kg. A embalagem foi identificada como rasgada, resultando na exposição do produto e necessidade de intervenção imediata. O volume foi segregado.</t>
+  </si>
+  <si>
+    <t>7022961</t>
+  </si>
+  <si>
+    <t>Durante movimentação interna, foi identificada a seguinte não conformidade física: A) O produto SPEED CANA SCX25KG (Lote 76181/26) apresentou avaria em 01 sacaria, totalizando 25kg. A embalagem foi identificada como rasgada, comprometendo a proteção do conteúdo e gerando vazamento no pallet. O volume foi imediatamente segregado.</t>
   </si>
 </sst>
 </file>
@@ -693,8 +714,8 @@
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="19.95" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="18" width="25.77734375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="25.77734375" style="1" hidden="1"/>
-    <col min="20" max="20" width="25.77734375" hidden="1"/>
+    <col min="19" max="19" width="25.77734375" style="1" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="25.77734375" hidden="1" customWidth="1"/>
     <col min="21" max="16384" width="25.77734375" style="1" hidden="1"/>
   </cols>
   <sheetData>
@@ -760,13 +781,13 @@
     </row>
     <row r="2" spans="1:20" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>19</v>
@@ -775,43 +796,43 @@
         <v>19</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H2" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="J2" s="10" t="s">
-        <v>31</v>
-      </c>
       <c r="K2" s="10" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="L2" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N2" s="13">
+        <v>25</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="R2" s="10" t="s">
         <v>37</v>
-      </c>
-      <c r="M2" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="N2" s="13">
-        <v>10</v>
-      </c>
-      <c r="O2" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="P2" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q2" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="R2" s="10" t="s">
-        <v>21</v>
       </c>
       <c r="S2" s="4">
         <f>IF(B2="",0,1)</f>
@@ -821,58 +842,58 @@
     </row>
     <row r="3" spans="1:20" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D3" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="10" t="s">
+      <c r="G3" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="10" t="s">
-        <v>40</v>
-      </c>
       <c r="H3" s="10" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="L3" s="10" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="M3" s="10" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="N3" s="13">
-        <v>1000</v>
+        <v>50</v>
       </c>
       <c r="O3" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P3" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="P3" s="10" t="s">
-        <v>46</v>
-      </c>
       <c r="Q3" s="10" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="S3" s="4">
         <f>IF(B3="",0,1)</f>
@@ -881,52 +902,124 @@
       <c r="T3"/>
     </row>
     <row r="4" spans="1:20" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
-      <c r="Q4" s="10"/>
-      <c r="R4" s="10"/>
+      <c r="A4" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="I4" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="N4" s="13">
+        <v>50</v>
+      </c>
+      <c r="O4" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q4" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="R4" s="10" t="s">
+        <v>37</v>
+      </c>
       <c r="S4" s="4">
         <f>IF(B4="",0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4"/>
     </row>
     <row r="5" spans="1:20" s="3" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="10"/>
+      <c r="A5" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="M5" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="N5" s="13">
+        <v>25</v>
+      </c>
+      <c r="O5" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="P5" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q5" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="R5" s="10" t="s">
+        <v>37</v>
+      </c>
       <c r="S5" s="4">
         <f t="shared" ref="S5:S12" si="0">IF(B5="",0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5"/>
     </row>
@@ -1133,11 +1226,11 @@
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="6" type="noConversion"/>
+  <conditionalFormatting sqref="I12:I13 I1">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I12:I13 I1">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L12:M1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="4"/>

</xml_diff>